<commit_message>
wip: snapshot of in-progress work before UX enhancements
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Input/SalesTeam.xlsx
+++ b/Input/SalesTeam.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\PowerBIData\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\07PREPORT\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8F20D9-5279-46DB-8FF0-6FCF3C4AE937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0D9E14B-B7C3-499F-9CC8-F046FFDD7E85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C5D50CEC-F3D4-4C64-AB24-EE3E368D105E}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{C5D50CEC-F3D4-4C64-AB24-EE3E368D105E}"/>
   </bookViews>
   <sheets>
     <sheet name="salesperson" sheetId="4" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="154">
   <si>
     <t>Company</t>
   </si>
@@ -493,9 +493,6 @@
     <t>Mohamed Abdulhady</t>
   </si>
   <si>
-    <t>Ahmed Mrajea</t>
-  </si>
-  <si>
     <t>kaled Alwani</t>
   </si>
   <si>
@@ -503,13 +500,19 @@
   </si>
   <si>
     <t>Yousef Salim</t>
+  </si>
+  <si>
+    <t>Ahmed Mandi</t>
+  </si>
+  <si>
+    <t>Ahmed Belgasim</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -952,15 +955,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC391F98-6EB3-4C23-89C7-B05415492034}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:D72"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:D73"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.88671875" customWidth="1"/>
     <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>123</v>
       </c>
@@ -974,7 +977,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:4" hidden="1">
+    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
@@ -988,7 +991,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
@@ -1002,7 +1005,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="4" spans="1:4" hidden="1">
+    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1016,12 +1019,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" spans="1:4" hidden="1">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" hidden="1">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
@@ -1035,12 +1038,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" spans="1:4" hidden="1">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:4" hidden="1">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>14</v>
       </c>
@@ -1054,7 +1057,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" spans="1:4" hidden="1">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1068,12 +1071,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="10" spans="1:4" hidden="1">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:4" hidden="1">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1084,17 +1087,17 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:4" hidden="1">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:4" hidden="1">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:4" hidden="1">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -1108,19 +1111,19 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" spans="1:4" hidden="1">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:4" hidden="1">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:4" hidden="1">
+    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B17" t="s">
         <v>106</v>
@@ -1132,12 +1135,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:4" hidden="1">
+    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:4" hidden="1">
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -1151,17 +1154,17 @@
         <v>145</v>
       </c>
     </row>
-    <row r="20" spans="1:4" hidden="1">
+    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:4" hidden="1">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:4" hidden="1">
+    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>124</v>
       </c>
@@ -1175,7 +1178,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="23" spans="1:4" hidden="1">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -1189,7 +1192,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="24" spans="1:4" hidden="1">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1203,12 +1206,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="25" spans="1:4" hidden="1">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:4" hidden="1">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -1222,22 +1225,22 @@
         <v>145</v>
       </c>
     </row>
-    <row r="27" spans="1:4" hidden="1">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:4" hidden="1">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:4" hidden="1">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:4" hidden="1">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -1251,7 +1254,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="31" spans="1:4" hidden="1">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -1265,7 +1268,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="32" spans="1:4" hidden="1">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>37</v>
       </c>
@@ -1279,7 +1282,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>38</v>
       </c>
@@ -1293,7 +1296,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="34" spans="1:4" hidden="1">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>39</v>
       </c>
@@ -1307,12 +1310,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="35" spans="1:4" hidden="1">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>41</v>
       </c>
@@ -1326,7 +1329,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>42</v>
       </c>
@@ -1340,12 +1343,12 @@
         <v>144</v>
       </c>
     </row>
-    <row r="38" spans="1:4" hidden="1">
+    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:4" hidden="1">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>44</v>
       </c>
@@ -1359,7 +1362,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="40" spans="1:4" hidden="1">
+    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>45</v>
       </c>
@@ -1373,12 +1376,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="41" spans="1:4" hidden="1">
+    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:4" hidden="1">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>47</v>
       </c>
@@ -1392,12 +1395,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="43" spans="1:4" hidden="1">
+    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:4" hidden="1">
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -1411,14 +1414,14 @@
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:4" hidden="1">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:4" hidden="1">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>111</v>
@@ -1430,7 +1433,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="47" spans="1:4" hidden="1">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -1444,12 +1447,12 @@
         <v>144</v>
       </c>
     </row>
-    <row r="48" spans="1:4" hidden="1">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="49" spans="1:4" hidden="1">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>53</v>
       </c>
@@ -1463,17 +1466,17 @@
         <v>145</v>
       </c>
     </row>
-    <row r="50" spans="1:4" hidden="1">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="51" spans="1:4" hidden="1">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="52" spans="1:4" hidden="1">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>56</v>
       </c>
@@ -1487,12 +1490,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="53" spans="1:4" hidden="1">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="54" spans="1:4" hidden="1">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>58</v>
       </c>
@@ -1500,12 +1503,12 @@
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:4" hidden="1">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="56" spans="1:4" hidden="1">
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>60</v>
       </c>
@@ -1519,22 +1522,22 @@
         <v>145</v>
       </c>
     </row>
-    <row r="57" spans="1:4" hidden="1">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="58" spans="1:4" hidden="1">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="59" spans="1:4" hidden="1">
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="60" spans="1:4" hidden="1">
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>140</v>
       </c>
@@ -1548,7 +1551,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="61" spans="1:4">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>64</v>
       </c>
@@ -1562,32 +1565,32 @@
         <v>144</v>
       </c>
     </row>
-    <row r="62" spans="1:4" hidden="1">
+    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="63" spans="1:4" hidden="1">
+    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="64" spans="1:4" hidden="1">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="65" spans="1:4" hidden="1">
+    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="66" spans="1:4" hidden="1">
+    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="67" spans="1:4" hidden="1">
+    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>138</v>
       </c>
@@ -1601,7 +1604,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="68" spans="1:4">
+    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>148</v>
       </c>
@@ -1615,7 +1618,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="69" spans="1:4">
+    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
         <v>30</v>
       </c>
@@ -1629,9 +1632,9 @@
         <v>143</v>
       </c>
     </row>
-    <row r="70" spans="1:4" hidden="1">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B70" t="s">
         <v>103</v>
@@ -1643,7 +1646,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="71" spans="1:4" hidden="1">
+    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>139</v>
       </c>
@@ -1657,9 +1660,9 @@
         <v>145</v>
       </c>
     </row>
-    <row r="72" spans="1:4" hidden="1">
+    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B72" t="s">
         <v>133</v>
@@ -1668,6 +1671,20 @@
         <v>100</v>
       </c>
       <c r="D72" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>153</v>
+      </c>
+      <c r="B73" t="s">
+        <v>103</v>
+      </c>
+      <c r="C73" t="s">
+        <v>100</v>
+      </c>
+      <c r="D73" t="s">
         <v>145</v>
       </c>
     </row>
@@ -1675,9 +1692,7 @@
   <autoFilter ref="A1:D72" xr:uid="{EC391F98-6EB3-4C23-89C7-B05415492034}">
     <filterColumn colId="1">
       <filters>
-        <filter val="TK-CNT-BB"/>
-        <filter val="TK-EST-BB"/>
-        <filter val="TK-WST-BB"/>
+        <filter val="MJ-BD-BC-01"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -1689,14 +1704,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC21A7DE-912C-4AFC-AA98-99DE924F1A47}">
   <dimension ref="A1:I28"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.109375" customWidth="1"/>
     <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="30.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>72</v>
       </c>
@@ -1719,7 +1734,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>118</v>
       </c>
@@ -1737,7 +1752,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>119</v>
       </c>
@@ -1760,7 +1775,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>120</v>
       </c>
@@ -1777,7 +1792,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>121</v>
       </c>
@@ -1794,7 +1809,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>122</v>
       </c>
@@ -1814,7 +1829,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>127</v>
       </c>
@@ -1831,7 +1846,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>103</v>
       </c>
@@ -1854,7 +1869,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>104</v>
       </c>
@@ -1877,7 +1892,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
         <v>130</v>
       </c>
@@ -1900,7 +1915,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
         <v>114</v>
       </c>
@@ -1923,7 +1938,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>141</v>
       </c>
@@ -1946,7 +1961,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>101</v>
       </c>
@@ -1969,7 +1984,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>102</v>
       </c>
@@ -1992,7 +2007,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>113</v>
       </c>
@@ -2012,7 +2027,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>105</v>
       </c>
@@ -2035,7 +2050,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
         <v>136</v>
       </c>
@@ -2056,7 +2071,7 @@
       </c>
       <c r="I17" s="2"/>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>126</v>
       </c>
@@ -2074,7 +2089,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
         <v>109</v>
       </c>
@@ -2097,7 +2112,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>117</v>
       </c>
@@ -2120,7 +2135,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>133</v>
       </c>
@@ -2143,7 +2158,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>112</v>
       </c>
@@ -2163,7 +2178,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>108</v>
       </c>
@@ -2183,7 +2198,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>111</v>
       </c>
@@ -2206,7 +2221,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>106</v>
       </c>
@@ -2229,7 +2244,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="13" t="s">
         <v>107</v>
       </c>
@@ -2252,7 +2267,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="25.8" customHeight="1">
+    <row r="27" spans="1:9" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>135</v>
       </c>
@@ -2275,7 +2290,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="22.2" customHeight="1">
+    <row r="28" spans="1:9" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="13" t="s">
         <v>110</v>
       </c>

</xml_diff>